<commit_message>
models tunning in progress
</commit_message>
<xml_diff>
--- a/description.xlsx
+++ b/description.xlsx
@@ -664,70 +664,70 @@
         <v>0.4168055555555555</v>
       </c>
       <c r="F3" t="n">
-        <v>0.08</v>
+        <v>0.08631944444444445</v>
       </c>
       <c r="G3" t="n">
-        <v>0.07597222222222222</v>
+        <v>0.08208333333333333</v>
       </c>
       <c r="H3" t="n">
-        <v>0.754375</v>
+        <v>1.039861111111111</v>
       </c>
       <c r="I3" t="n">
-        <v>0.08</v>
+        <v>0.08631944444444445</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6743749999999999</v>
+        <v>0.9535416666666666</v>
       </c>
       <c r="K3" t="n">
-        <v>1.230625</v>
+        <v>0.994375</v>
       </c>
       <c r="L3" t="n">
-        <v>2.765902777777778</v>
+        <v>3.005625</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9927083333333333</v>
+        <v>1.098194444444444</v>
       </c>
       <c r="N3" t="n">
-        <v>9.199361111111111</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O3" t="n">
-        <v>9.199361111111111</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="P3" t="n">
-        <v>9.199361111111111</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.59933333333333</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R3" t="n">
-        <v>61.59744068287036</v>
+        <v>60.01405671296295</v>
       </c>
       <c r="S3" t="n">
-        <v>65.23410734953704</v>
+        <v>62.48426649305556</v>
       </c>
       <c r="T3" t="n">
-        <v>68.23589265046296</v>
+        <v>66.14869791666668</v>
       </c>
       <c r="U3" t="n">
-        <v>73.77899305555556</v>
+        <v>69.43722077546296</v>
       </c>
       <c r="V3" t="n">
-        <v>2.001685474537036</v>
+        <v>2.075224247685184</v>
       </c>
       <c r="W3" t="n">
-        <v>1.820001446759258</v>
+        <v>1.960923032407406</v>
       </c>
       <c r="X3" t="n">
-        <v>1.653291377314814</v>
+        <v>1.770920138888888</v>
       </c>
       <c r="Y3" t="n">
-        <v>1.427777777777778</v>
+        <v>1.604542824074073</v>
       </c>
       <c r="Z3" t="n">
-        <v>6.902756076388886</v>
+        <v>7.411610243055551</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.270625</v>
+        <v>0.3175694444444445</v>
       </c>
     </row>
     <row r="4">
@@ -749,70 +749,70 @@
         <v>0.4930472249694865</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2713026197184134</v>
+        <v>0.2808449310699747</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4343797521449056</v>
+        <v>0.4530132694449632</v>
       </c>
       <c r="H4" t="n">
-        <v>1.233663984444602</v>
+        <v>1.599081263637332</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2713026197184134</v>
+        <v>0.2808449310699747</v>
       </c>
       <c r="J4" t="n">
-        <v>1.202474021397949</v>
+        <v>1.574545758335848</v>
       </c>
       <c r="K4" t="n">
-        <v>1.23790332315364</v>
+        <v>1.145821432718675</v>
       </c>
       <c r="L4" t="n">
-        <v>1.237475858641897</v>
+        <v>1.145821432718675</v>
       </c>
       <c r="M4" t="n">
-        <v>3.971688074158616</v>
+        <v>4.196681602369729</v>
       </c>
       <c r="N4" t="n">
-        <v>0.07666666666666661</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>0.07666666666666661</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>0.07666666666666661</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.07999999999999996</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>28.8515878081365</v>
+        <v>28.45611528951303</v>
       </c>
       <c r="S4" t="n">
-        <v>29.57150406635467</v>
+        <v>28.97670720505194</v>
       </c>
       <c r="T4" t="n">
-        <v>30.08558313617703</v>
+        <v>29.59086422309393</v>
       </c>
       <c r="U4" t="n">
-        <v>29.80035649097718</v>
+        <v>29.73474374798742</v>
       </c>
       <c r="V4" t="n">
-        <v>0.8882650710623478</v>
+        <v>0.8157094799286484</v>
       </c>
       <c r="W4" t="n">
-        <v>1.023761520335448</v>
+        <v>0.9235176523660829</v>
       </c>
       <c r="X4" t="n">
-        <v>1.108026837109246</v>
+        <v>1.052021016241708</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.237336405860896</v>
+        <v>1.126830814857516</v>
       </c>
       <c r="Z4" t="n">
-        <v>2.958528596833556</v>
+        <v>2.665214046230623</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.519609863792214</v>
+        <v>1.646744825639112</v>
       </c>
     </row>
     <row r="5">
@@ -858,16 +858,16 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -952,19 +952,19 @@
         <v>9.199999999999999</v>
       </c>
       <c r="Q6" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R6" t="n">
-        <v>36.95833333333333</v>
+        <v>35.93749999999999</v>
       </c>
       <c r="S6" t="n">
-        <v>39.77083333333334</v>
+        <v>37.74999999999999</v>
       </c>
       <c r="T6" t="n">
-        <v>42.33333333333334</v>
+        <v>40.75</v>
       </c>
       <c r="U6" t="n">
-        <v>49</v>
+        <v>43.9375</v>
       </c>
       <c r="V6" t="n">
         <v>2.395833333333329</v>
@@ -979,7 +979,7 @@
         <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>4.791666666666664</v>
+        <v>4.791666666666671</v>
       </c>
       <c r="AA6" t="n">
         <v>0</v>
@@ -1037,19 +1037,19 @@
         <v>9.199999999999999</v>
       </c>
       <c r="Q7" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R7" t="n">
-        <v>62.89583333333335</v>
+        <v>60.89583333333335</v>
       </c>
       <c r="S7" t="n">
-        <v>68.12500000000003</v>
+        <v>64.10416666666669</v>
       </c>
       <c r="T7" t="n">
-        <v>73.875</v>
+        <v>69.68750000000001</v>
       </c>
       <c r="U7" t="n">
-        <v>87</v>
+        <v>75.79166666666667</v>
       </c>
       <c r="V7" t="n">
         <v>2.395833333333332</v>
@@ -1061,10 +1061,10 @@
         <v>2.395833333333329</v>
       </c>
       <c r="Y7" t="n">
-        <v>2.5</v>
+        <v>2.395833333333329</v>
       </c>
       <c r="Z7" t="n">
-        <v>7.291666666666661</v>
+        <v>9.583333333333314</v>
       </c>
       <c r="AA7" t="n">
         <v>0</v>
@@ -1122,16 +1122,16 @@
         <v>9.199999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>88.68749999999997</v>
+        <v>85.68749999999999</v>
       </c>
       <c r="S8" t="n">
-        <v>96.66666666666663</v>
+        <v>90.27083333333331</v>
       </c>
       <c r="T8" t="n">
-        <v>100</v>
+        <v>99.64583333333329</v>
       </c>
       <c r="U8" t="n">
         <v>100</v>
@@ -1146,10 +1146,10 @@
         <v>2.395833333333336</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.5</v>
+        <v>2.395833333333336</v>
       </c>
       <c r="Z8" t="n">
-        <v>9.687499999999993</v>
+        <v>9.583333333333329</v>
       </c>
       <c r="AA8" t="n">
         <v>0</v>
@@ -1180,13 +1180,13 @@
         <v>7</v>
       </c>
       <c r="H9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K9" t="n">
         <v>4</v>
@@ -1207,7 +1207,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="Q9" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="R9" t="n">
         <v>102.25</v>
@@ -1219,7 +1219,7 @@
         <v>102.25</v>
       </c>
       <c r="U9" t="n">
-        <v>102</v>
+        <v>102.25</v>
       </c>
       <c r="V9" t="n">
         <v>2.395833333333336</v>
@@ -1231,13 +1231,13 @@
         <v>2.395833333333336</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.5</v>
+        <v>2.395833333333336</v>
       </c>
       <c r="Z9" t="n">
-        <v>9.687500000000007</v>
+        <v>9.583333333333343</v>
       </c>
       <c r="AA9" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>